<commit_message>
Fixed duplicate file processing
</commit_message>
<xml_diff>
--- a/AEF_files copy - do not touch/10.syntax.passed/202504251541---Thailand AEF_2023.syntax_checked.xlsx
+++ b/AEF_files copy - do not touch/10.syntax.passed/202504251541---Thailand AEF_2023.syntax_checked.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unfccc365.sharepoint.com/sites/Mitigation/Paris Agreement Article 6/Article 6.2/03_CARP/consistency/AEF_files copy/10.syntax.passed/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unfccc365.sharepoint.com/sites/Mitigation/Paris Agreement Article 6/Article 6.2/03_CARP/consistency/AEF_files copy - do not touch/10.syntax.passed/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="3" documentId="11_AC3361E587CDCD3B09DC6E2D90397F84A8E6C737" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C74A9738-B0E9-0D4E-93D8-6B25B75159A7}"/>
   <bookViews>
-    <workbookView xWindow="7080" yWindow="9800" windowWidth="38460" windowHeight="17720" tabRatio="618" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7080" yWindow="9740" windowWidth="38460" windowHeight="17720" tabRatio="618" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Index" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,20 @@
     <definedName name="Transfer">#REF!</definedName>
     <definedName name="Use">#REF!</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -4437,8 +4450,53 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008FB6730B0802B54A9F00C78B857E1443" ma:contentTypeVersion="21" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e758502e7902c92bdb050e89a8fea950">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="819ae873-75e1-413b-9d00-7af9258cf281" xmlns:ns3="eb4559c4-8463-4985-927f-f0d558bff8f0" xmlns:ns4="13d80b15-5f07-43ab-b435-85767a7dac08" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f4060acd4b29e25a8a76462245842ebf" ns2:_="" ns3:_="" ns4:_="">
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="819ae873-75e1-413b-9d00-7af9258cf281">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="eb4559c4-8463-4985-927f-f0d558bff8f0" xsi:nil="true"/>
+    <Ready xmlns="819ae873-75e1-413b-9d00-7af9258cf281">true</Ready>
+    <Doc_x002e_SymbolNumber xmlns="819ae873-75e1-413b-9d00-7af9258cf281" xsi:nil="true"/>
+    <_Flow_SignoffStatus xmlns="819ae873-75e1-413b-9d00-7af9258cf281" xsi:nil="true"/>
+    <Formatter_x0028_s_x0029_ xmlns="819ae873-75e1-413b-9d00-7af9258cf281">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Formatter_x0028_s_x0029_>
+    <Status xmlns="819ae873-75e1-413b-9d00-7af9258cf281">true</Status>
+    <Teamleademail xmlns="819ae873-75e1-413b-9d00-7af9258cf281">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Teamleademail>
+    <Drafter_x0028_s_x0029_ xmlns="819ae873-75e1-413b-9d00-7af9258cf281">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Drafter_x0028_s_x0029_>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008FB6730B0802B54A9F00C78B857E1443" ma:contentTypeVersion="28" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9d684dda10f4f2dbf746fae76444930a">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="819ae873-75e1-413b-9d00-7af9258cf281" xmlns:ns3="eb4559c4-8463-4985-927f-f0d558bff8f0" xmlns:ns4="13d80b15-5f07-43ab-b435-85767a7dac08" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2e1a7d6f560f2b9324fa8d4f4f1cd31a" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="819ae873-75e1-413b-9d00-7af9258cf281"/>
     <xsd:import namespace="eb4559c4-8463-4985-927f-f0d558bff8f0"/>
     <xsd:import namespace="13d80b15-5f07-43ab-b435-85767a7dac08"/>
@@ -4465,9 +4523,12 @@
                 <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:Comments" minOccurs="0"/>
                 <xsd:element ref="ns2:Ready" minOccurs="0"/>
                 <xsd:element ref="ns2:_Flow_SignoffStatus" minOccurs="0"/>
+                <xsd:element ref="ns2:Teamleademail" minOccurs="0"/>
+                <xsd:element ref="ns2:Drafter_x0028_s_x0029_" minOccurs="0"/>
+                <xsd:element ref="ns2:Formatter_x0028_s_x0029_" minOccurs="0"/>
+                <xsd:element ref="ns2:Status" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -4556,21 +4617,81 @@
         <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="Comments" ma:index="26" nillable="true" ma:displayName="Comments" ma:format="Dropdown" ma:internalName="Comments">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="Ready" ma:index="27" nillable="true" ma:displayName="Ready" ma:default="1" ma:format="Dropdown" ma:internalName="Ready">
+    <xsd:element name="Ready" ma:index="26" nillable="true" ma:displayName="Ready" ma:default="1" ma:format="Dropdown" ma:internalName="Ready">
       <xsd:simpleType>
         <xsd:restriction base="dms:Boolean"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="_Flow_SignoffStatus" ma:index="28" nillable="true" ma:displayName="Sign-off status" ma:internalName="_x0024_Resources_x003a_core_x002c_Signoff_Status">
+    <xsd:element name="_Flow_SignoffStatus" ma:index="27" nillable="true" ma:displayName="Sign-off status" ma:format="Dropdown" ma:internalName="_x0024_Resources_x003a_core_x002c_Signoff_Status">
       <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
+        <xsd:restriction base="dms:Choice">
+          <xsd:enumeration value="WIP"/>
+          <xsd:enumeration value="Ready for clearance"/>
+          <xsd:enumeration value="Cleared"/>
+          <xsd:enumeration value="Returned"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="Teamleademail" ma:index="28" nillable="true" ma:displayName="Team lead(s)" ma:format="Dropdown" ma:list="UserInfo" ma:SharePointGroup="0" ma:internalName="Teamleademail">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="Drafter_x0028_s_x0029_" ma:index="29" nillable="true" ma:displayName="Drafter(s)" ma:format="Dropdown" ma:list="UserInfo" ma:SharePointGroup="0" ma:internalName="Drafter_x0028_s_x0029_">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="Formatter_x0028_s_x0029_" ma:index="30" nillable="true" ma:displayName="Formatter(s)" ma:format="Dropdown" ma:list="UserInfo" ma:SharePointGroup="0" ma:internalName="Formatter_x0028_s_x0029_">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:User">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="Status" ma:index="31" nillable="true" ma:displayName="Status" ma:default="1" ma:format="Dropdown" ma:internalName="Status">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Boolean"/>
       </xsd:simpleType>
     </xsd:element>
   </xsd:schema>
@@ -4718,51 +4839,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="819ae873-75e1-413b-9d00-7af9258cf281">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="eb4559c4-8463-4985-927f-f0d558bff8f0" xsi:nil="true"/>
-    <Ready xmlns="819ae873-75e1-413b-9d00-7af9258cf281">true</Ready>
-    <Comments xmlns="819ae873-75e1-413b-9d00-7af9258cf281" xsi:nil="true"/>
-    <Doc_x002e_SymbolNumber xmlns="819ae873-75e1-413b-9d00-7af9258cf281" xsi:nil="true"/>
-    <_Flow_SignoffStatus xmlns="819ae873-75e1-413b-9d00-7af9258cf281" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="9d8c265a-5436-43a7-80c1-713d2827ffde" ContentTypeId="0x0101" PreviousValue="false"/>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0E1FDC6E-B636-4FE0-B398-EB528D8067CE}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A9799D65-07E5-48E8-AA39-49E0191F739B}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="819ae873-75e1-413b-9d00-7af9258cf281"/>
-    <ds:schemaRef ds:uri="eb4559c4-8463-4985-927f-f0d558bff8f0"/>
-    <ds:schemaRef ds:uri="13d80b15-5f07-43ab-b435-85767a7dac08"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -4770,27 +4855,23 @@
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F09D9509-AE1F-4384-AA74-2A606E86234E}">
   <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="819ae873-75e1-413b-9d00-7af9258cf281"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="eb4559c4-8463-4985-927f-f0d558bff8f0"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
     <ds:schemaRef ds:uri="13d80b15-5f07-43ab-b435-85767a7dac08"/>
-    <ds:schemaRef ds:uri="eb4559c4-8463-4985-927f-f0d558bff8f0"/>
-    <ds:schemaRef ds:uri="819ae873-75e1-413b-9d00-7af9258cf281"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A9799D65-07E5-48E8-AA39-49E0191F739B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{205112EA-5000-4529-A6DA-0F2977C327AA}"/>
 </file>
 
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>